<commit_message>
fix bug not full volcabulary
</commit_message>
<xml_diff>
--- a/volcabulary.xlsx
+++ b/volcabulary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\work\kocogi621998.github.io\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F11E80E9-4D77-424E-AC72-D73F1D0A82D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{DB7933BC-513A-4CBB-860B-1E4061FEDBB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2295" yWindow="2295" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19388,16 +19388,16 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -23319,1082 +23319,1082 @@
       <c r="Z114" s="1"/>
     </row>
     <row r="115" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A115" s="4" t="s">
+      <c r="A115" s="5" t="s">
         <v>683</v>
       </c>
-      <c r="B115" s="4" t="s">
+      <c r="B115" s="5" t="s">
         <v>684</v>
       </c>
-      <c r="C115" s="4" t="s">
+      <c r="C115" s="5" t="s">
         <v>860</v>
       </c>
-      <c r="D115" s="4" t="s">
+      <c r="D115" s="5" t="s">
         <v>861</v>
       </c>
-      <c r="E115" s="4" t="s">
+      <c r="E115" s="5" t="s">
         <v>685</v>
       </c>
-      <c r="F115" s="5" t="s">
+      <c r="F115" s="4" t="s">
         <v>686</v>
       </c>
     </row>
     <row r="116" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A116" s="4" t="s">
+      <c r="A116" s="5" t="s">
         <v>687</v>
       </c>
-      <c r="B116" s="4" t="s">
+      <c r="B116" s="5" t="s">
         <v>688</v>
       </c>
-      <c r="C116" s="4" t="s">
+      <c r="C116" s="5" t="s">
         <v>862</v>
       </c>
-      <c r="D116" s="4" t="s">
+      <c r="D116" s="5" t="s">
         <v>863</v>
       </c>
-      <c r="E116" s="4" t="s">
+      <c r="E116" s="5" t="s">
         <v>689</v>
       </c>
-      <c r="F116" s="5" t="s">
+      <c r="F116" s="4" t="s">
         <v>864</v>
       </c>
     </row>
     <row r="117" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A117" s="4" t="s">
+      <c r="A117" s="5" t="s">
         <v>690</v>
       </c>
-      <c r="B117" s="4" t="s">
+      <c r="B117" s="5" t="s">
         <v>691</v>
       </c>
-      <c r="C117" s="4" t="s">
+      <c r="C117" s="5" t="s">
         <v>865</v>
       </c>
-      <c r="D117" s="4" t="s">
+      <c r="D117" s="5" t="s">
         <v>866</v>
       </c>
-      <c r="E117" s="4" t="s">
+      <c r="E117" s="5" t="s">
         <v>692</v>
       </c>
-      <c r="F117" s="5" t="s">
+      <c r="F117" s="4" t="s">
         <v>693</v>
       </c>
     </row>
     <row r="118" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A118" s="4" t="s">
+      <c r="A118" s="5" t="s">
         <v>694</v>
       </c>
-      <c r="B118" s="4" t="s">
+      <c r="B118" s="5" t="s">
         <v>695</v>
       </c>
-      <c r="C118" s="4" t="s">
+      <c r="C118" s="5" t="s">
         <v>867</v>
       </c>
-      <c r="D118" s="4" t="s">
+      <c r="D118" s="5" t="s">
         <v>868</v>
       </c>
-      <c r="E118" s="4" t="s">
+      <c r="E118" s="5" t="s">
         <v>696</v>
       </c>
-      <c r="F118" s="5" t="s">
+      <c r="F118" s="4" t="s">
         <v>869</v>
       </c>
     </row>
     <row r="119" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A119" s="4" t="s">
+      <c r="A119" s="5" t="s">
         <v>697</v>
       </c>
-      <c r="B119" s="4" t="s">
+      <c r="B119" s="5" t="s">
         <v>698</v>
       </c>
-      <c r="C119" s="4" t="s">
+      <c r="C119" s="5" t="s">
         <v>870</v>
       </c>
-      <c r="D119" s="4" t="s">
+      <c r="D119" s="5" t="s">
         <v>871</v>
       </c>
-      <c r="E119" s="4" t="s">
+      <c r="E119" s="5" t="s">
         <v>699</v>
       </c>
-      <c r="F119" s="5" t="s">
+      <c r="F119" s="4" t="s">
         <v>700</v>
       </c>
     </row>
     <row r="120" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A120" s="4" t="s">
+      <c r="A120" s="5" t="s">
         <v>701</v>
       </c>
-      <c r="B120" s="4" t="s">
+      <c r="B120" s="5" t="s">
         <v>702</v>
       </c>
-      <c r="C120" s="4" t="s">
+      <c r="C120" s="5" t="s">
         <v>872</v>
       </c>
-      <c r="D120" s="4" t="s">
+      <c r="D120" s="5" t="s">
         <v>873</v>
       </c>
-      <c r="E120" s="4" t="s">
+      <c r="E120" s="5" t="s">
         <v>703</v>
       </c>
-      <c r="F120" s="5" t="s">
+      <c r="F120" s="4" t="s">
         <v>704</v>
       </c>
     </row>
     <row r="121" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A121" s="4" t="s">
+      <c r="A121" s="5" t="s">
         <v>705</v>
       </c>
-      <c r="B121" s="4" t="s">
+      <c r="B121" s="5" t="s">
         <v>706</v>
       </c>
-      <c r="C121" s="4" t="s">
+      <c r="C121" s="5" t="s">
         <v>874</v>
       </c>
-      <c r="D121" s="4" t="s">
+      <c r="D121" s="5" t="s">
         <v>875</v>
       </c>
-      <c r="E121" s="4" t="s">
+      <c r="E121" s="5" t="s">
         <v>707</v>
       </c>
-      <c r="F121" s="5" t="s">
+      <c r="F121" s="4" t="s">
         <v>876</v>
       </c>
     </row>
     <row r="122" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A122" s="4" t="s">
+      <c r="A122" s="5" t="s">
         <v>708</v>
       </c>
-      <c r="B122" s="4" t="s">
+      <c r="B122" s="5" t="s">
         <v>709</v>
       </c>
-      <c r="C122" s="4" t="s">
+      <c r="C122" s="5" t="s">
         <v>877</v>
       </c>
-      <c r="D122" s="4" t="s">
+      <c r="D122" s="5" t="s">
         <v>878</v>
       </c>
-      <c r="E122" s="4" t="s">
+      <c r="E122" s="5" t="s">
         <v>710</v>
       </c>
-      <c r="F122" s="5" t="s">
+      <c r="F122" s="4" t="s">
         <v>879</v>
       </c>
     </row>
     <row r="123" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A123" s="4" t="s">
+      <c r="A123" s="5" t="s">
         <v>711</v>
       </c>
-      <c r="B123" s="4" t="s">
+      <c r="B123" s="5" t="s">
         <v>712</v>
       </c>
-      <c r="C123" s="4" t="s">
+      <c r="C123" s="5" t="s">
         <v>880</v>
       </c>
-      <c r="D123" s="4" t="s">
+      <c r="D123" s="5" t="s">
         <v>881</v>
       </c>
-      <c r="E123" s="4" t="s">
+      <c r="E123" s="5" t="s">
         <v>713</v>
       </c>
-      <c r="F123" s="5" t="s">
+      <c r="F123" s="4" t="s">
         <v>882</v>
       </c>
     </row>
     <row r="124" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A124" s="4" t="s">
+      <c r="A124" s="5" t="s">
         <v>714</v>
       </c>
-      <c r="B124" s="4" t="s">
+      <c r="B124" s="5" t="s">
         <v>715</v>
       </c>
-      <c r="C124" s="4" t="s">
+      <c r="C124" s="5" t="s">
         <v>883</v>
       </c>
-      <c r="D124" s="4" t="s">
+      <c r="D124" s="5" t="s">
         <v>884</v>
       </c>
-      <c r="E124" s="4" t="s">
+      <c r="E124" s="5" t="s">
         <v>716</v>
       </c>
-      <c r="F124" s="5" t="s">
+      <c r="F124" s="4" t="s">
         <v>885</v>
       </c>
     </row>
     <row r="125" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A125" s="4" t="s">
+      <c r="A125" s="5" t="s">
         <v>717</v>
       </c>
-      <c r="B125" s="4" t="s">
+      <c r="B125" s="5" t="s">
         <v>718</v>
       </c>
-      <c r="C125" s="4" t="s">
+      <c r="C125" s="5" t="s">
         <v>886</v>
       </c>
-      <c r="D125" s="4" t="s">
+      <c r="D125" s="5" t="s">
         <v>887</v>
       </c>
-      <c r="E125" s="4" t="s">
+      <c r="E125" s="5" t="s">
         <v>719</v>
       </c>
-      <c r="F125" s="5" t="s">
+      <c r="F125" s="4" t="s">
         <v>888</v>
       </c>
     </row>
     <row r="126" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A126" s="4" t="s">
+      <c r="A126" s="5" t="s">
         <v>720</v>
       </c>
-      <c r="B126" s="4" t="s">
+      <c r="B126" s="5" t="s">
         <v>721</v>
       </c>
-      <c r="C126" s="4" t="s">
+      <c r="C126" s="5" t="s">
         <v>889</v>
       </c>
-      <c r="D126" s="4" t="s">
+      <c r="D126" s="5" t="s">
         <v>890</v>
       </c>
-      <c r="E126" s="4" t="s">
+      <c r="E126" s="5" t="s">
         <v>722</v>
       </c>
-      <c r="F126" s="5" t="s">
+      <c r="F126" s="4" t="s">
         <v>723</v>
       </c>
     </row>
     <row r="127" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A127" s="4" t="s">
+      <c r="A127" s="5" t="s">
         <v>724</v>
       </c>
-      <c r="B127" s="4" t="s">
+      <c r="B127" s="5" t="s">
         <v>725</v>
       </c>
-      <c r="C127" s="4" t="s">
+      <c r="C127" s="5" t="s">
         <v>891</v>
       </c>
-      <c r="D127" s="4" t="s">
+      <c r="D127" s="5" t="s">
         <v>892</v>
       </c>
-      <c r="E127" s="4" t="s">
+      <c r="E127" s="5" t="s">
         <v>726</v>
       </c>
-      <c r="F127" s="5" t="s">
+      <c r="F127" s="4" t="s">
         <v>727</v>
       </c>
     </row>
     <row r="128" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A128" s="4" t="s">
+      <c r="A128" s="5" t="s">
         <v>728</v>
       </c>
-      <c r="B128" s="4" t="s">
+      <c r="B128" s="5" t="s">
         <v>729</v>
       </c>
-      <c r="C128" s="4" t="s">
+      <c r="C128" s="5" t="s">
         <v>893</v>
       </c>
-      <c r="D128" s="4" t="s">
+      <c r="D128" s="5" t="s">
         <v>894</v>
       </c>
-      <c r="E128" s="4" t="s">
+      <c r="E128" s="5" t="s">
         <v>730</v>
       </c>
-      <c r="F128" s="5" t="s">
+      <c r="F128" s="4" t="s">
         <v>895</v>
       </c>
     </row>
     <row r="129" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A129" s="4" t="s">
+      <c r="A129" s="5" t="s">
         <v>731</v>
       </c>
-      <c r="B129" s="4" t="s">
+      <c r="B129" s="5" t="s">
         <v>732</v>
       </c>
-      <c r="C129" s="4" t="s">
+      <c r="C129" s="5" t="s">
         <v>896</v>
       </c>
-      <c r="D129" s="4" t="s">
+      <c r="D129" s="5" t="s">
         <v>897</v>
       </c>
-      <c r="E129" s="4" t="s">
+      <c r="E129" s="5" t="s">
         <v>733</v>
       </c>
-      <c r="F129" s="5" t="s">
+      <c r="F129" s="4" t="s">
         <v>898</v>
       </c>
     </row>
     <row r="130" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A130" s="4" t="s">
+      <c r="A130" s="5" t="s">
         <v>734</v>
       </c>
-      <c r="B130" s="4" t="s">
+      <c r="B130" s="5" t="s">
         <v>735</v>
       </c>
-      <c r="C130" s="4" t="s">
+      <c r="C130" s="5" t="s">
         <v>899</v>
       </c>
-      <c r="D130" s="4" t="s">
+      <c r="D130" s="5" t="s">
         <v>900</v>
       </c>
-      <c r="E130" s="4" t="s">
+      <c r="E130" s="5" t="s">
         <v>736</v>
       </c>
-      <c r="F130" s="4" t="s">
+      <c r="F130" s="5" t="s">
         <v>901</v>
       </c>
     </row>
     <row r="131" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A131" s="4" t="s">
+      <c r="A131" s="5" t="s">
         <v>737</v>
       </c>
-      <c r="B131" s="4" t="s">
+      <c r="B131" s="5" t="s">
         <v>738</v>
       </c>
-      <c r="C131" s="4" t="s">
+      <c r="C131" s="5" t="s">
         <v>902</v>
       </c>
-      <c r="D131" s="4" t="s">
+      <c r="D131" s="5" t="s">
         <v>903</v>
       </c>
-      <c r="E131" s="4" t="s">
+      <c r="E131" s="5" t="s">
         <v>739</v>
       </c>
-      <c r="F131" s="5" t="s">
+      <c r="F131" s="4" t="s">
         <v>904</v>
       </c>
     </row>
     <row r="132" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A132" s="4" t="s">
+      <c r="A132" s="5" t="s">
         <v>740</v>
       </c>
-      <c r="B132" s="4" t="s">
+      <c r="B132" s="5" t="s">
         <v>741</v>
       </c>
-      <c r="C132" s="4" t="s">
+      <c r="C132" s="5" t="s">
         <v>905</v>
       </c>
-      <c r="D132" s="4" t="s">
+      <c r="D132" s="5" t="s">
         <v>906</v>
       </c>
-      <c r="E132" s="4" t="s">
+      <c r="E132" s="5" t="s">
         <v>742</v>
       </c>
-      <c r="F132" s="5" t="s">
+      <c r="F132" s="4" t="s">
         <v>907</v>
       </c>
     </row>
     <row r="133" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A133" s="4" t="s">
+      <c r="A133" s="5" t="s">
         <v>743</v>
       </c>
-      <c r="B133" s="4" t="s">
+      <c r="B133" s="5" t="s">
         <v>744</v>
       </c>
-      <c r="C133" s="4" t="s">
+      <c r="C133" s="5" t="s">
         <v>908</v>
       </c>
-      <c r="D133" s="4" t="s">
+      <c r="D133" s="5" t="s">
         <v>909</v>
       </c>
-      <c r="E133" s="4" t="s">
+      <c r="E133" s="5" t="s">
         <v>745</v>
       </c>
-      <c r="F133" s="5" t="s">
+      <c r="F133" s="4" t="s">
         <v>910</v>
       </c>
     </row>
     <row r="134" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A134" s="4" t="s">
+      <c r="A134" s="5" t="s">
         <v>746</v>
       </c>
-      <c r="B134" s="4" t="s">
+      <c r="B134" s="5" t="s">
         <v>747</v>
       </c>
-      <c r="C134" s="4" t="s">
+      <c r="C134" s="5" t="s">
         <v>911</v>
       </c>
-      <c r="D134" s="4" t="s">
+      <c r="D134" s="5" t="s">
         <v>912</v>
       </c>
-      <c r="E134" s="4" t="s">
+      <c r="E134" s="5" t="s">
         <v>748</v>
       </c>
-      <c r="F134" s="5" t="s">
+      <c r="F134" s="4" t="s">
         <v>749</v>
       </c>
     </row>
     <row r="135" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A135" s="4" t="s">
+      <c r="A135" s="5" t="s">
         <v>750</v>
       </c>
-      <c r="B135" s="4" t="s">
+      <c r="B135" s="5" t="s">
         <v>751</v>
       </c>
-      <c r="C135" s="4" t="s">
+      <c r="C135" s="5" t="s">
         <v>913</v>
       </c>
-      <c r="D135" s="4" t="s">
+      <c r="D135" s="5" t="s">
         <v>914</v>
       </c>
-      <c r="E135" s="4" t="s">
+      <c r="E135" s="5" t="s">
         <v>752</v>
       </c>
-      <c r="F135" s="4" t="s">
+      <c r="F135" s="5" t="s">
         <v>915</v>
       </c>
     </row>
     <row r="136" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A136" s="4" t="s">
+      <c r="A136" s="5" t="s">
         <v>753</v>
       </c>
-      <c r="B136" s="4" t="s">
+      <c r="B136" s="5" t="s">
         <v>754</v>
       </c>
-      <c r="C136" s="4" t="s">
+      <c r="C136" s="5" t="s">
         <v>916</v>
       </c>
-      <c r="D136" s="4" t="s">
+      <c r="D136" s="5" t="s">
         <v>917</v>
       </c>
-      <c r="E136" s="4" t="s">
+      <c r="E136" s="5" t="s">
         <v>755</v>
       </c>
-      <c r="F136" s="5" t="s">
+      <c r="F136" s="4" t="s">
         <v>918</v>
       </c>
     </row>
     <row r="137" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A137" s="4" t="s">
+      <c r="A137" s="5" t="s">
         <v>756</v>
       </c>
-      <c r="B137" s="4" t="s">
+      <c r="B137" s="5" t="s">
         <v>757</v>
       </c>
-      <c r="C137" s="4" t="s">
+      <c r="C137" s="5" t="s">
         <v>919</v>
       </c>
-      <c r="D137" s="4" t="s">
+      <c r="D137" s="5" t="s">
         <v>920</v>
       </c>
-      <c r="E137" s="4" t="s">
+      <c r="E137" s="5" t="s">
         <v>758</v>
       </c>
-      <c r="F137" s="5" t="s">
+      <c r="F137" s="4" t="s">
         <v>921</v>
       </c>
     </row>
     <row r="138" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A138" s="4" t="s">
+      <c r="A138" s="5" t="s">
         <v>759</v>
       </c>
-      <c r="B138" s="4" t="s">
+      <c r="B138" s="5" t="s">
         <v>760</v>
       </c>
-      <c r="C138" s="4" t="s">
+      <c r="C138" s="5" t="s">
         <v>922</v>
       </c>
-      <c r="D138" s="4" t="s">
+      <c r="D138" s="5" t="s">
         <v>923</v>
       </c>
-      <c r="E138" s="4" t="s">
+      <c r="E138" s="5" t="s">
         <v>761</v>
       </c>
-      <c r="F138" s="5" t="s">
+      <c r="F138" s="4" t="s">
         <v>924</v>
       </c>
     </row>
     <row r="139" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A139" s="4" t="s">
+      <c r="A139" s="5" t="s">
         <v>762</v>
       </c>
-      <c r="B139" s="4" t="s">
+      <c r="B139" s="5" t="s">
         <v>763</v>
       </c>
-      <c r="C139" s="4" t="s">
+      <c r="C139" s="5" t="s">
         <v>925</v>
       </c>
-      <c r="D139" s="4" t="s">
+      <c r="D139" s="5" t="s">
         <v>926</v>
       </c>
-      <c r="E139" s="4" t="s">
+      <c r="E139" s="5" t="s">
         <v>764</v>
       </c>
-      <c r="F139" s="5" t="s">
+      <c r="F139" s="4" t="s">
         <v>927</v>
       </c>
     </row>
     <row r="140" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A140" s="4" t="s">
+      <c r="A140" s="5" t="s">
         <v>765</v>
       </c>
-      <c r="B140" s="4" t="s">
+      <c r="B140" s="5" t="s">
         <v>766</v>
       </c>
-      <c r="C140" s="4" t="s">
+      <c r="C140" s="5" t="s">
         <v>928</v>
       </c>
-      <c r="D140" s="4" t="s">
+      <c r="D140" s="5" t="s">
         <v>929</v>
       </c>
-      <c r="E140" s="4" t="s">
+      <c r="E140" s="5" t="s">
         <v>767</v>
       </c>
-      <c r="F140" s="5" t="s">
+      <c r="F140" s="4" t="s">
         <v>768</v>
       </c>
     </row>
     <row r="141" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A141" s="4" t="s">
+      <c r="A141" s="5" t="s">
         <v>769</v>
       </c>
-      <c r="B141" s="4" t="s">
+      <c r="B141" s="5" t="s">
         <v>770</v>
       </c>
-      <c r="C141" s="4" t="s">
+      <c r="C141" s="5" t="s">
         <v>930</v>
       </c>
-      <c r="D141" s="4" t="s">
+      <c r="D141" s="5" t="s">
         <v>931</v>
       </c>
-      <c r="E141" s="4" t="s">
+      <c r="E141" s="5" t="s">
         <v>771</v>
       </c>
-      <c r="F141" s="5" t="s">
+      <c r="F141" s="4" t="s">
         <v>932</v>
       </c>
     </row>
     <row r="142" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A142" s="4" t="s">
+      <c r="A142" s="5" t="s">
         <v>772</v>
       </c>
-      <c r="B142" s="4" t="s">
+      <c r="B142" s="5" t="s">
         <v>773</v>
       </c>
-      <c r="C142" s="4" t="s">
+      <c r="C142" s="5" t="s">
         <v>933</v>
       </c>
-      <c r="D142" s="4" t="s">
+      <c r="D142" s="5" t="s">
         <v>934</v>
       </c>
-      <c r="E142" s="4" t="s">
+      <c r="E142" s="5" t="s">
         <v>774</v>
       </c>
-      <c r="F142" s="5" t="s">
+      <c r="F142" s="4" t="s">
         <v>935</v>
       </c>
     </row>
     <row r="143" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A143" s="4" t="s">
+      <c r="A143" s="5" t="s">
         <v>775</v>
       </c>
-      <c r="B143" s="4" t="s">
+      <c r="B143" s="5" t="s">
         <v>776</v>
       </c>
-      <c r="C143" s="4" t="s">
+      <c r="C143" s="5" t="s">
         <v>936</v>
       </c>
-      <c r="D143" s="4" t="s">
+      <c r="D143" s="5" t="s">
         <v>937</v>
       </c>
-      <c r="E143" s="4" t="s">
+      <c r="E143" s="5" t="s">
         <v>777</v>
       </c>
-      <c r="F143" s="5" t="s">
+      <c r="F143" s="4" t="s">
         <v>938</v>
       </c>
     </row>
     <row r="144" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A144" s="4" t="s">
+      <c r="A144" s="5" t="s">
         <v>778</v>
       </c>
-      <c r="B144" s="4" t="s">
+      <c r="B144" s="5" t="s">
         <v>779</v>
       </c>
-      <c r="C144" s="4" t="s">
+      <c r="C144" s="5" t="s">
         <v>939</v>
       </c>
-      <c r="D144" s="4" t="s">
+      <c r="D144" s="5" t="s">
         <v>940</v>
       </c>
-      <c r="E144" s="4" t="s">
+      <c r="E144" s="5" t="s">
         <v>780</v>
       </c>
-      <c r="F144" s="5" t="s">
+      <c r="F144" s="4" t="s">
         <v>781</v>
       </c>
     </row>
     <row r="145" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A145" s="4" t="s">
+      <c r="A145" s="5" t="s">
         <v>782</v>
       </c>
-      <c r="B145" s="4" t="s">
+      <c r="B145" s="5" t="s">
         <v>783</v>
       </c>
-      <c r="C145" s="4" t="s">
+      <c r="C145" s="5" t="s">
         <v>941</v>
       </c>
-      <c r="D145" s="4" t="s">
+      <c r="D145" s="5" t="s">
         <v>942</v>
       </c>
-      <c r="E145" s="4" t="s">
+      <c r="E145" s="5" t="s">
         <v>784</v>
       </c>
-      <c r="F145" s="5" t="s">
+      <c r="F145" s="4" t="s">
         <v>943</v>
       </c>
     </row>
     <row r="146" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A146" s="4" t="s">
+      <c r="A146" s="5" t="s">
         <v>785</v>
       </c>
-      <c r="B146" s="4" t="s">
+      <c r="B146" s="5" t="s">
         <v>786</v>
       </c>
-      <c r="C146" s="4" t="s">
+      <c r="C146" s="5" t="s">
         <v>944</v>
       </c>
-      <c r="D146" s="4" t="s">
+      <c r="D146" s="5" t="s">
         <v>945</v>
       </c>
-      <c r="E146" s="4" t="s">
+      <c r="E146" s="5" t="s">
         <v>787</v>
       </c>
-      <c r="F146" s="5" t="s">
+      <c r="F146" s="4" t="s">
         <v>946</v>
       </c>
     </row>
     <row r="147" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A147" s="4" t="s">
+      <c r="A147" s="5" t="s">
         <v>788</v>
       </c>
-      <c r="B147" s="4" t="s">
+      <c r="B147" s="5" t="s">
         <v>789</v>
       </c>
-      <c r="C147" s="4" t="s">
+      <c r="C147" s="5" t="s">
         <v>947</v>
       </c>
-      <c r="D147" s="4" t="s">
+      <c r="D147" s="5" t="s">
         <v>948</v>
       </c>
-      <c r="E147" s="4" t="s">
+      <c r="E147" s="5" t="s">
         <v>790</v>
       </c>
-      <c r="F147" s="5" t="s">
+      <c r="F147" s="4" t="s">
         <v>949</v>
       </c>
     </row>
     <row r="148" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A148" s="4" t="s">
+      <c r="A148" s="5" t="s">
         <v>791</v>
       </c>
-      <c r="B148" s="4" t="s">
+      <c r="B148" s="5" t="s">
         <v>792</v>
       </c>
-      <c r="C148" s="4" t="s">
+      <c r="C148" s="5" t="s">
         <v>950</v>
       </c>
-      <c r="D148" s="4" t="s">
+      <c r="D148" s="5" t="s">
         <v>951</v>
       </c>
-      <c r="E148" s="4" t="s">
+      <c r="E148" s="5" t="s">
         <v>793</v>
       </c>
-      <c r="F148" s="5" t="s">
+      <c r="F148" s="4" t="s">
         <v>952</v>
       </c>
     </row>
     <row r="149" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A149" s="4" t="s">
+      <c r="A149" s="5" t="s">
         <v>794</v>
       </c>
-      <c r="B149" s="4" t="s">
+      <c r="B149" s="5" t="s">
         <v>795</v>
       </c>
-      <c r="C149" s="4" t="s">
+      <c r="C149" s="5" t="s">
         <v>953</v>
       </c>
-      <c r="D149" s="4" t="s">
+      <c r="D149" s="5" t="s">
         <v>954</v>
       </c>
-      <c r="E149" s="4" t="s">
+      <c r="E149" s="5" t="s">
         <v>796</v>
       </c>
-      <c r="F149" s="5" t="s">
+      <c r="F149" s="4" t="s">
         <v>797</v>
       </c>
     </row>
     <row r="150" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A150" s="4" t="s">
+      <c r="A150" s="5" t="s">
         <v>798</v>
       </c>
-      <c r="B150" s="4" t="s">
+      <c r="B150" s="5" t="s">
         <v>799</v>
       </c>
-      <c r="C150" s="4" t="s">
+      <c r="C150" s="5" t="s">
         <v>955</v>
       </c>
-      <c r="D150" s="4" t="s">
+      <c r="D150" s="5" t="s">
         <v>956</v>
       </c>
-      <c r="E150" s="4" t="s">
+      <c r="E150" s="5" t="s">
         <v>800</v>
       </c>
-      <c r="F150" s="5" t="s">
+      <c r="F150" s="4" t="s">
         <v>957</v>
       </c>
     </row>
     <row r="151" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A151" s="4" t="s">
+      <c r="A151" s="5" t="s">
         <v>801</v>
       </c>
-      <c r="B151" s="4" t="s">
+      <c r="B151" s="5" t="s">
         <v>802</v>
       </c>
-      <c r="C151" s="4" t="s">
+      <c r="C151" s="5" t="s">
         <v>958</v>
       </c>
-      <c r="D151" s="4" t="s">
+      <c r="D151" s="5" t="s">
         <v>959</v>
       </c>
-      <c r="E151" s="4" t="s">
+      <c r="E151" s="5" t="s">
         <v>803</v>
       </c>
-      <c r="F151" s="5" t="s">
+      <c r="F151" s="4" t="s">
         <v>960</v>
       </c>
     </row>
     <row r="152" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A152" s="4" t="s">
+      <c r="A152" s="5" t="s">
         <v>804</v>
       </c>
-      <c r="B152" s="4" t="s">
+      <c r="B152" s="5" t="s">
         <v>805</v>
       </c>
-      <c r="C152" s="4" t="s">
+      <c r="C152" s="5" t="s">
         <v>961</v>
       </c>
-      <c r="D152" s="4" t="s">
+      <c r="D152" s="5" t="s">
         <v>962</v>
       </c>
-      <c r="E152" s="4" t="s">
+      <c r="E152" s="5" t="s">
         <v>806</v>
       </c>
-      <c r="F152" s="5" t="s">
+      <c r="F152" s="4" t="s">
         <v>807</v>
       </c>
     </row>
     <row r="153" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A153" s="4" t="s">
+      <c r="A153" s="5" t="s">
         <v>808</v>
       </c>
-      <c r="B153" s="4" t="s">
+      <c r="B153" s="5" t="s">
         <v>809</v>
       </c>
-      <c r="C153" s="4" t="s">
+      <c r="C153" s="5" t="s">
         <v>963</v>
       </c>
-      <c r="D153" s="4" t="s">
+      <c r="D153" s="5" t="s">
         <v>964</v>
       </c>
-      <c r="E153" s="4" t="s">
+      <c r="E153" s="5" t="s">
         <v>810</v>
       </c>
-      <c r="F153" s="5" t="s">
+      <c r="F153" s="4" t="s">
         <v>811</v>
       </c>
     </row>
     <row r="154" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A154" s="4" t="s">
+      <c r="A154" s="5" t="s">
         <v>812</v>
       </c>
-      <c r="B154" s="4" t="s">
+      <c r="B154" s="5" t="s">
         <v>813</v>
       </c>
-      <c r="C154" s="4" t="s">
+      <c r="C154" s="5" t="s">
         <v>965</v>
       </c>
-      <c r="D154" s="4" t="s">
+      <c r="D154" s="5" t="s">
         <v>966</v>
       </c>
-      <c r="E154" s="4" t="s">
+      <c r="E154" s="5" t="s">
         <v>814</v>
       </c>
-      <c r="F154" s="5" t="s">
+      <c r="F154" s="4" t="s">
         <v>815</v>
       </c>
     </row>
     <row r="155" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A155" s="4" t="s">
+      <c r="A155" s="5" t="s">
         <v>816</v>
       </c>
-      <c r="B155" s="4" t="s">
+      <c r="B155" s="5" t="s">
         <v>817</v>
       </c>
-      <c r="C155" s="4" t="s">
+      <c r="C155" s="5" t="s">
         <v>967</v>
       </c>
-      <c r="D155" s="4" t="s">
+      <c r="D155" s="5" t="s">
         <v>968</v>
       </c>
-      <c r="E155" s="4" t="s">
+      <c r="E155" s="5" t="s">
         <v>818</v>
       </c>
-      <c r="F155" s="5" t="s">
+      <c r="F155" s="4" t="s">
         <v>819</v>
       </c>
     </row>
     <row r="156" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A156" s="4" t="s">
+      <c r="A156" s="5" t="s">
         <v>820</v>
       </c>
-      <c r="B156" s="4" t="s">
+      <c r="B156" s="5" t="s">
         <v>821</v>
       </c>
-      <c r="C156" s="4" t="s">
+      <c r="C156" s="5" t="s">
         <v>969</v>
       </c>
-      <c r="D156" s="4" t="s">
+      <c r="D156" s="5" t="s">
         <v>970</v>
       </c>
-      <c r="E156" s="4" t="s">
+      <c r="E156" s="5" t="s">
         <v>822</v>
       </c>
-      <c r="F156" s="5" t="s">
+      <c r="F156" s="4" t="s">
         <v>971</v>
       </c>
     </row>
     <row r="157" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A157" s="4" t="s">
+      <c r="A157" s="5" t="s">
         <v>823</v>
       </c>
-      <c r="B157" s="4" t="s">
+      <c r="B157" s="5" t="s">
         <v>824</v>
       </c>
-      <c r="C157" s="4" t="s">
+      <c r="C157" s="5" t="s">
         <v>972</v>
       </c>
-      <c r="D157" s="4" t="s">
+      <c r="D157" s="5" t="s">
         <v>973</v>
       </c>
-      <c r="E157" s="4" t="s">
+      <c r="E157" s="5" t="s">
         <v>825</v>
       </c>
-      <c r="F157" s="5" t="s">
+      <c r="F157" s="4" t="s">
         <v>974</v>
       </c>
     </row>
     <row r="158" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A158" s="4" t="s">
+      <c r="A158" s="5" t="s">
         <v>826</v>
       </c>
-      <c r="B158" s="4" t="s">
+      <c r="B158" s="5" t="s">
         <v>827</v>
       </c>
-      <c r="C158" s="4" t="s">
+      <c r="C158" s="5" t="s">
         <v>975</v>
       </c>
-      <c r="D158" s="4" t="s">
+      <c r="D158" s="5" t="s">
         <v>976</v>
       </c>
-      <c r="E158" s="4" t="s">
+      <c r="E158" s="5" t="s">
         <v>828</v>
       </c>
-      <c r="F158" s="4" t="s">
+      <c r="F158" s="5" t="s">
         <v>977</v>
       </c>
     </row>
     <row r="159" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A159" s="4" t="s">
+      <c r="A159" s="5" t="s">
         <v>829</v>
       </c>
-      <c r="B159" s="4" t="s">
+      <c r="B159" s="5" t="s">
         <v>830</v>
       </c>
-      <c r="C159" s="4" t="s">
+      <c r="C159" s="5" t="s">
         <v>978</v>
       </c>
-      <c r="D159" s="4" t="s">
+      <c r="D159" s="5" t="s">
         <v>979</v>
       </c>
-      <c r="E159" s="4" t="s">
+      <c r="E159" s="5" t="s">
         <v>831</v>
       </c>
-      <c r="F159" s="5" t="s">
+      <c r="F159" s="4" t="s">
         <v>832</v>
       </c>
     </row>
     <row r="160" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A160" s="4" t="s">
+      <c r="A160" s="5" t="s">
         <v>833</v>
       </c>
-      <c r="B160" s="4" t="s">
+      <c r="B160" s="5" t="s">
         <v>834</v>
       </c>
-      <c r="C160" s="4" t="s">
+      <c r="C160" s="5" t="s">
         <v>980</v>
       </c>
-      <c r="D160" s="4" t="s">
+      <c r="D160" s="5" t="s">
         <v>981</v>
       </c>
-      <c r="E160" s="4" t="s">
+      <c r="E160" s="5" t="s">
         <v>835</v>
       </c>
-      <c r="F160" s="5" t="s">
+      <c r="F160" s="4" t="s">
         <v>982</v>
       </c>
     </row>
     <row r="161" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A161" s="4" t="s">
+      <c r="A161" s="5" t="s">
         <v>836</v>
       </c>
-      <c r="B161" s="4" t="s">
+      <c r="B161" s="5" t="s">
         <v>837</v>
       </c>
-      <c r="C161" s="4" t="s">
+      <c r="C161" s="5" t="s">
         <v>983</v>
       </c>
-      <c r="D161" s="4" t="s">
+      <c r="D161" s="5" t="s">
         <v>984</v>
       </c>
-      <c r="E161" s="4" t="s">
+      <c r="E161" s="5" t="s">
         <v>838</v>
       </c>
-      <c r="F161" s="5" t="s">
+      <c r="F161" s="4" t="s">
         <v>985</v>
       </c>
     </row>
     <row r="162" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A162" s="4" t="s">
+      <c r="A162" s="5" t="s">
         <v>839</v>
       </c>
-      <c r="B162" s="4" t="s">
+      <c r="B162" s="5" t="s">
         <v>840</v>
       </c>
-      <c r="C162" s="4" t="s">
+      <c r="C162" s="5" t="s">
         <v>986</v>
       </c>
-      <c r="D162" s="4" t="s">
+      <c r="D162" s="5" t="s">
         <v>987</v>
       </c>
-      <c r="E162" s="4" t="s">
+      <c r="E162" s="5" t="s">
         <v>841</v>
       </c>
-      <c r="F162" s="5" t="s">
+      <c r="F162" s="4" t="s">
         <v>988</v>
       </c>
     </row>
     <row r="163" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A163" s="4" t="s">
+      <c r="A163" s="5" t="s">
         <v>842</v>
       </c>
-      <c r="B163" s="4" t="s">
+      <c r="B163" s="5" t="s">
         <v>843</v>
       </c>
-      <c r="C163" s="4" t="s">
+      <c r="C163" s="5" t="s">
         <v>989</v>
       </c>
-      <c r="D163" s="4" t="s">
+      <c r="D163" s="5" t="s">
         <v>990</v>
       </c>
-      <c r="E163" s="4" t="s">
+      <c r="E163" s="5" t="s">
         <v>844</v>
       </c>
-      <c r="F163" s="5" t="s">
+      <c r="F163" s="4" t="s">
         <v>991</v>
       </c>
     </row>
     <row r="164" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A164" s="4" t="s">
+      <c r="A164" s="5" t="s">
         <v>845</v>
       </c>
-      <c r="B164" s="4" t="s">
+      <c r="B164" s="5" t="s">
         <v>846</v>
       </c>
-      <c r="C164" s="4" t="s">
+      <c r="C164" s="5" t="s">
         <v>992</v>
       </c>
-      <c r="D164" s="4" t="s">
+      <c r="D164" s="5" t="s">
         <v>993</v>
       </c>
-      <c r="E164" s="4" t="s">
+      <c r="E164" s="5" t="s">
         <v>847</v>
       </c>
-      <c r="F164" s="5" t="s">
+      <c r="F164" s="4" t="s">
         <v>994</v>
       </c>
     </row>
     <row r="165" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A165" s="4" t="s">
+      <c r="A165" s="5" t="s">
         <v>848</v>
       </c>
-      <c r="B165" s="4" t="s">
+      <c r="B165" s="5" t="s">
         <v>849</v>
       </c>
-      <c r="C165" s="4" t="s">
+      <c r="C165" s="5" t="s">
         <v>995</v>
       </c>
-      <c r="D165" s="4" t="s">
+      <c r="D165" s="5" t="s">
         <v>996</v>
       </c>
-      <c r="E165" s="4" t="s">
+      <c r="E165" s="5" t="s">
         <v>850</v>
       </c>
-      <c r="F165" s="5" t="s">
+      <c r="F165" s="4" t="s">
         <v>997</v>
       </c>
     </row>
     <row r="166" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A166" s="4" t="s">
+      <c r="A166" s="5" t="s">
         <v>851</v>
       </c>
-      <c r="B166" s="4" t="s">
+      <c r="B166" s="5" t="s">
         <v>852</v>
       </c>
-      <c r="C166" s="4" t="s">
+      <c r="C166" s="5" t="s">
         <v>998</v>
       </c>
-      <c r="D166" s="4" t="s">
+      <c r="D166" s="5" t="s">
         <v>999</v>
       </c>
-      <c r="E166" s="4" t="s">
+      <c r="E166" s="5" t="s">
         <v>853</v>
       </c>
-      <c r="F166" s="5" t="s">
+      <c r="F166" s="4" t="s">
         <v>1000</v>
       </c>
     </row>
     <row r="167" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A167" s="4" t="s">
+      <c r="A167" s="5" t="s">
         <v>854</v>
       </c>
-      <c r="B167" s="4" t="s">
+      <c r="B167" s="5" t="s">
         <v>855</v>
       </c>
-      <c r="C167" s="4" t="s">
+      <c r="C167" s="5" t="s">
         <v>1001</v>
       </c>
-      <c r="D167" s="4" t="s">
+      <c r="D167" s="5" t="s">
         <v>1002</v>
       </c>
-      <c r="E167" s="4" t="s">
+      <c r="E167" s="5" t="s">
         <v>856</v>
       </c>
-      <c r="F167" s="5" t="s">
+      <c r="F167" s="4" t="s">
         <v>1003</v>
       </c>
     </row>
     <row r="168" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A168" s="4" t="s">
+      <c r="A168" s="5" t="s">
         <v>857</v>
       </c>
-      <c r="B168" s="4" t="s">
+      <c r="B168" s="5" t="s">
         <v>858</v>
       </c>
-      <c r="C168" s="4" t="s">
+      <c r="C168" s="5" t="s">
         <v>1004</v>
       </c>
-      <c r="D168" s="4" t="s">
+      <c r="D168" s="5" t="s">
         <v>1005</v>
       </c>
-      <c r="E168" s="4" t="s">
+      <c r="E168" s="5" t="s">
         <v>859</v>
       </c>
-      <c r="F168" s="5" t="s">
+      <c r="F168" s="4" t="s">
         <v>1006</v>
       </c>
     </row>

</xml_diff>